<commit_message>
Support OLICATI temario import format
</commit_message>
<xml_diff>
--- a/docs/imports/machote_temarios.xlsx
+++ b/docs/imports/machote_temarios.xlsx
@@ -15,30 +15,42 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="18">
   <si>
     <t>Nombre de la materia</t>
   </si>
   <si>
+    <t>Creditos</t>
+  </si>
+  <si>
+    <t>Objetivo general</t>
+  </si>
+  <si>
     <t>Objetivo general del curso</t>
   </si>
   <si>
-    <t>Creditos</t>
-  </si>
-  <si>
     <t>1. Nombre de la unidad</t>
   </si>
   <si>
     <t>Objetivo especifico de la unidad</t>
   </si>
   <si>
+    <t>conceptual</t>
+  </si>
+  <si>
     <t>1.1. Nombre del tema</t>
   </si>
   <si>
     <t>1.1.1. Nombre del subtema</t>
   </si>
   <si>
+    <t>procedimental</t>
+  </si>
+  <si>
     <t>1.1.2. Nombre del subtema</t>
+  </si>
+  <si>
+    <t>actitudinal</t>
   </si>
   <si>
     <t>1.2. Nombre del tema</t>
@@ -409,96 +421,158 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="true" style="0"/>
     <col min="2" max="2" width="80" customWidth="true" style="0"/>
+    <col min="3" max="3" width="18" customWidth="true" style="0"/>
+    <col min="4" max="4" width="18" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
       </c>
       <c r="B2" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3"/>
-      <c r="B3"/>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="2" t="s">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2"/>
-    </row>
-    <row r="6" spans="1:2">
+      <c r="C5" s="2">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2"/>
-    </row>
-    <row r="7" spans="1:2">
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" s="2"/>
-    </row>
-    <row r="8" spans="1:2">
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B8" s="2"/>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="C8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="2"/>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="2" t="s">
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2">
         <v>10</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="2"/>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="2"/>
+      <c r="D14" s="2"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>